<commit_message>
Corregir estado en vivo y llave final
</commit_message>
<xml_diff>
--- a/src/resultados_partidos.xlsx
+++ b/src/resultados_partidos.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1720" uniqueCount="371">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1744" uniqueCount="379">
   <si>
     <t>id</t>
   </si>
@@ -988,112 +988,136 @@
     <t>03/07/2026</t>
   </si>
   <si>
+    <t>3 de julio</t>
+  </si>
+  <si>
+    <t>20:30</t>
+  </si>
+  <si>
+    <t>3/07/2026</t>
+  </si>
+  <si>
+    <t>Colombia vs Ghana</t>
+  </si>
+  <si>
+    <t>13:00</t>
+  </si>
+  <si>
+    <t>Australia vs Egipto</t>
+  </si>
+  <si>
+    <t>Argentina vs Cabo Verde</t>
+  </si>
+  <si>
+    <t>R16</t>
+  </si>
+  <si>
+    <t>04/07/2026</t>
+  </si>
+  <si>
+    <t>4 de julio</t>
+  </si>
+  <si>
+    <t>4/07/2026</t>
+  </si>
+  <si>
+    <t>Paraguay vs Francia</t>
+  </si>
+  <si>
+    <t>Canadá vs Marruecos</t>
+  </si>
+  <si>
+    <t>05/07/2026</t>
+  </si>
+  <si>
+    <t>5 de julio</t>
+  </si>
+  <si>
+    <t>5/07/2026</t>
+  </si>
+  <si>
+    <t>Brasil vs Noruega</t>
+  </si>
+  <si>
+    <t>México vs Inglaterra</t>
+  </si>
+  <si>
+    <t>06/07/2026</t>
+  </si>
+  <si>
+    <t>6 de julio</t>
+  </si>
+  <si>
+    <t>6/07/2026</t>
+  </si>
+  <si>
+    <t>Portugal vs España</t>
+  </si>
+  <si>
+    <t>Estados Unidos vs Bélgica</t>
+  </si>
+  <si>
+    <t>07/07/2026</t>
+  </si>
+  <si>
+    <t>in_progress</t>
+  </si>
+  <si>
+    <t>7 de julio</t>
+  </si>
+  <si>
+    <t>7/07/2026</t>
+  </si>
+  <si>
+    <t>En vivo</t>
+  </si>
+  <si>
+    <t>Argentina vs Egipto</t>
+  </si>
+  <si>
     <t>scheduled</t>
   </si>
   <si>
-    <t>3 de julio</t>
-  </si>
-  <si>
-    <t>20:30</t>
-  </si>
-  <si>
-    <t>3/07/2026</t>
-  </si>
-  <si>
     <t>Por jugar</t>
   </si>
   <si>
-    <t>Colombia vs Ghana</t>
-  </si>
-  <si>
-    <t>13:00</t>
-  </si>
-  <si>
-    <t>Australia vs Egipto</t>
-  </si>
-  <si>
-    <t>Argentina vs Cabo Verde</t>
-  </si>
-  <si>
-    <t>R16</t>
-  </si>
-  <si>
-    <t>04/07/2026</t>
-  </si>
-  <si>
-    <t>4 de julio</t>
-  </si>
-  <si>
-    <t>4/07/2026</t>
-  </si>
-  <si>
-    <t>Paraguay vs Francia</t>
-  </si>
-  <si>
-    <t>Canadá vs Marruecos</t>
-  </si>
-  <si>
-    <t>05/07/2026</t>
-  </si>
-  <si>
-    <t>5 de julio</t>
-  </si>
-  <si>
-    <t>5/07/2026</t>
-  </si>
-  <si>
-    <t>Brasil vs Noruega</t>
-  </si>
-  <si>
-    <t>México vs Inglaterra</t>
-  </si>
-  <si>
-    <t>06/07/2026</t>
-  </si>
-  <si>
-    <t>6 de julio</t>
-  </si>
-  <si>
-    <t>6/07/2026</t>
+    <t>Suiza vs Colombia</t>
+  </si>
+  <si>
+    <t>QF</t>
+  </si>
+  <si>
+    <t>09/07/2026</t>
+  </si>
+  <si>
+    <t>9 de julio</t>
+  </si>
+  <si>
+    <t>9/07/2026</t>
+  </si>
+  <si>
+    <t>Francia vs Marruecos</t>
+  </si>
+  <si>
+    <t>10/07/2026</t>
+  </si>
+  <si>
+    <t>10 de julio</t>
+  </si>
+  <si>
+    <t>España vs Bélgica</t>
+  </si>
+  <si>
+    <t>11/07/2026</t>
+  </si>
+  <si>
+    <t>11 de julio</t>
+  </si>
+  <si>
+    <t>Noruega vs Inglaterra</t>
   </si>
   <si>
     <t>Por definir vs Por definir</t>
-  </si>
-  <si>
-    <t>Estados Unidos vs Bélgica</t>
-  </si>
-  <si>
-    <t>07/07/2026</t>
-  </si>
-  <si>
-    <t>7 de julio</t>
-  </si>
-  <si>
-    <t>7/07/2026</t>
-  </si>
-  <si>
-    <t>QF</t>
-  </si>
-  <si>
-    <t>09/07/2026</t>
-  </si>
-  <si>
-    <t>9 de julio</t>
-  </si>
-  <si>
-    <t>9/07/2026</t>
-  </si>
-  <si>
-    <t>10/07/2026</t>
-  </si>
-  <si>
-    <t>10 de julio</t>
-  </si>
-  <si>
-    <t>11/07/2026</t>
-  </si>
-  <si>
-    <t>11 de julio</t>
   </si>
   <si>
     <t>SF</t>
@@ -8256,30 +8280,34 @@
       <c r="Q87" s="2" t="s">
         <v>323</v>
       </c>
-      <c r="R87" s="1"/>
-      <c r="S87" s="1"/>
+      <c r="R87" s="1">
+        <v>1</v>
+      </c>
+      <c r="S87" s="1">
+        <v>0</v>
+      </c>
       <c r="T87" s="1"/>
       <c r="U87" s="1"/>
       <c r="V87" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="W87" s="2" t="s">
         <v>324</v>
       </c>
-      <c r="W87" s="2" t="s">
+      <c r="X87" s="2" t="s">
         <v>325</v>
       </c>
-      <c r="X87" s="2" t="s">
+      <c r="Y87" s="2" t="s">
         <v>326</v>
       </c>
-      <c r="Y87" s="2" t="s">
+      <c r="Z87" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="AA87" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="AB87" s="2" t="s">
         <v>327</v>
-      </c>
-      <c r="Z87" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="AA87" s="2" t="s">
-        <v>328</v>
-      </c>
-      <c r="AB87" s="2" t="s">
-        <v>329</v>
       </c>
     </row>
     <row r="88" spans="1:28">
@@ -8329,13 +8357,13 @@
         <v>323</v>
       </c>
       <c r="R88" s="1">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="S88" s="1">
         <v>1</v>
       </c>
       <c r="T88" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="U88" s="1">
         <v>4</v>
@@ -8344,13 +8372,13 @@
         <v>38</v>
       </c>
       <c r="W88" s="2" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="X88" s="2" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="Y88" s="2" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="Z88" s="2" t="s">
         <v>300</v>
@@ -8359,7 +8387,7 @@
         <v>154</v>
       </c>
       <c r="AB88" s="2" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
     </row>
     <row r="89" spans="1:28">
@@ -8420,13 +8448,13 @@
         <v>38</v>
       </c>
       <c r="W89" s="2" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="X89" s="2" t="s">
         <v>88</v>
       </c>
       <c r="Y89" s="2" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="Z89" s="2" t="s">
         <v>315</v>
@@ -8435,7 +8463,7 @@
         <v>185</v>
       </c>
       <c r="AB89" s="2" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
     </row>
     <row r="90" spans="1:28">
@@ -8446,7 +8474,7 @@
         <v>90</v>
       </c>
       <c r="C90" s="2" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="D90" s="2"/>
       <c r="E90" s="1">
@@ -8482,32 +8510,36 @@
         <v>65</v>
       </c>
       <c r="Q90" s="2" t="s">
-        <v>334</v>
-      </c>
-      <c r="R90" s="1"/>
-      <c r="S90" s="1"/>
+        <v>332</v>
+      </c>
+      <c r="R90" s="1">
+        <v>0</v>
+      </c>
+      <c r="S90" s="1">
+        <v>1</v>
+      </c>
       <c r="T90" s="1"/>
       <c r="U90" s="1"/>
       <c r="V90" s="2" t="s">
-        <v>324</v>
+        <v>38</v>
       </c>
       <c r="W90" s="2" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="X90" s="2" t="s">
         <v>251</v>
       </c>
       <c r="Y90" s="2" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="Z90" s="2" t="s">
         <v>41</v>
       </c>
       <c r="AA90" s="2" t="s">
-        <v>328</v>
+        <v>172</v>
       </c>
       <c r="AB90" s="2" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
     </row>
     <row r="91" spans="1:28">
@@ -8518,7 +8550,7 @@
         <v>89</v>
       </c>
       <c r="C91" s="2" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="D91" s="2"/>
       <c r="E91" s="1">
@@ -8554,32 +8586,36 @@
         <v>65</v>
       </c>
       <c r="Q91" s="2" t="s">
-        <v>334</v>
-      </c>
-      <c r="R91" s="1"/>
-      <c r="S91" s="1"/>
+        <v>332</v>
+      </c>
+      <c r="R91" s="1">
+        <v>0</v>
+      </c>
+      <c r="S91" s="1">
+        <v>3</v>
+      </c>
       <c r="T91" s="1"/>
       <c r="U91" s="1"/>
       <c r="V91" s="2" t="s">
-        <v>324</v>
+        <v>38</v>
       </c>
       <c r="W91" s="2" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="X91" s="2" t="s">
         <v>114</v>
       </c>
       <c r="Y91" s="2" t="s">
+        <v>334</v>
+      </c>
+      <c r="Z91" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="AA91" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="AB91" s="2" t="s">
         <v>336</v>
-      </c>
-      <c r="Z91" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="AA91" s="2" t="s">
-        <v>328</v>
-      </c>
-      <c r="AB91" s="2" t="s">
-        <v>338</v>
       </c>
     </row>
     <row r="92" spans="1:28">
@@ -8590,7 +8626,7 @@
         <v>91</v>
       </c>
       <c r="C92" s="2" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="D92" s="2"/>
       <c r="E92" s="1">
@@ -8626,32 +8662,36 @@
         <v>65</v>
       </c>
       <c r="Q92" s="2" t="s">
-        <v>339</v>
-      </c>
-      <c r="R92" s="1"/>
-      <c r="S92" s="1"/>
+        <v>337</v>
+      </c>
+      <c r="R92" s="1">
+        <v>1</v>
+      </c>
+      <c r="S92" s="1">
+        <v>2</v>
+      </c>
       <c r="T92" s="1"/>
       <c r="U92" s="1"/>
       <c r="V92" s="2" t="s">
-        <v>324</v>
+        <v>38</v>
       </c>
       <c r="W92" s="2" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="X92" s="2" t="s">
         <v>123</v>
       </c>
       <c r="Y92" s="2" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="Z92" s="2" t="s">
         <v>41</v>
       </c>
       <c r="AA92" s="2" t="s">
-        <v>328</v>
+        <v>181</v>
       </c>
       <c r="AB92" s="2" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
     </row>
     <row r="93" spans="1:28">
@@ -8662,7 +8702,7 @@
         <v>92</v>
       </c>
       <c r="C93" s="2" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="D93" s="2"/>
       <c r="E93" s="1">
@@ -8698,32 +8738,36 @@
         <v>36</v>
       </c>
       <c r="Q93" s="2" t="s">
-        <v>339</v>
-      </c>
-      <c r="R93" s="1"/>
-      <c r="S93" s="1"/>
+        <v>337</v>
+      </c>
+      <c r="R93" s="1">
+        <v>2</v>
+      </c>
+      <c r="S93" s="1">
+        <v>3</v>
+      </c>
       <c r="T93" s="1"/>
       <c r="U93" s="1"/>
       <c r="V93" s="2" t="s">
-        <v>324</v>
+        <v>38</v>
       </c>
       <c r="W93" s="2" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="X93" s="2" t="s">
-        <v>239</v>
+        <v>70</v>
       </c>
       <c r="Y93" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="Z93" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="AA93" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="AB93" s="2" t="s">
         <v>341</v>
-      </c>
-      <c r="Z93" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="AA93" s="2" t="s">
-        <v>328</v>
-      </c>
-      <c r="AB93" s="2" t="s">
-        <v>343</v>
       </c>
     </row>
     <row r="94" spans="1:28">
@@ -8734,16 +8778,28 @@
         <v>93</v>
       </c>
       <c r="C94" s="2" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="D94" s="2"/>
-      <c r="E94" s="1"/>
-      <c r="F94" s="2"/>
-      <c r="G94" s="2"/>
+      <c r="E94" s="1">
+        <v>41</v>
+      </c>
+      <c r="F94" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="G94" s="2" t="s">
+        <v>199</v>
+      </c>
       <c r="H94" s="2"/>
-      <c r="I94" s="1"/>
-      <c r="J94" s="2"/>
-      <c r="K94" s="2"/>
+      <c r="I94" s="1">
+        <v>30</v>
+      </c>
+      <c r="J94" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="K94" s="2" t="s">
+        <v>142</v>
+      </c>
       <c r="L94" s="2"/>
       <c r="M94" s="1">
         <v>2</v>
@@ -8758,32 +8814,36 @@
         <v>65</v>
       </c>
       <c r="Q94" s="2" t="s">
-        <v>344</v>
-      </c>
-      <c r="R94" s="1"/>
-      <c r="S94" s="1"/>
+        <v>342</v>
+      </c>
+      <c r="R94" s="1">
+        <v>0</v>
+      </c>
+      <c r="S94" s="1">
+        <v>1</v>
+      </c>
       <c r="T94" s="1"/>
       <c r="U94" s="1"/>
       <c r="V94" s="2" t="s">
-        <v>324</v>
+        <v>38</v>
       </c>
       <c r="W94" s="2" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="X94" s="2" t="s">
         <v>40</v>
       </c>
       <c r="Y94" s="2" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="Z94" s="2" t="s">
         <v>41</v>
       </c>
       <c r="AA94" s="2" t="s">
-        <v>328</v>
+        <v>141</v>
       </c>
       <c r="AB94" s="2" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
     </row>
     <row r="95" spans="1:28">
@@ -8794,7 +8854,7 @@
         <v>94</v>
       </c>
       <c r="C95" s="2" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="D95" s="2"/>
       <c r="E95" s="1">
@@ -8830,32 +8890,36 @@
         <v>65</v>
       </c>
       <c r="Q95" s="2" t="s">
-        <v>344</v>
-      </c>
-      <c r="R95" s="1"/>
-      <c r="S95" s="1"/>
+        <v>342</v>
+      </c>
+      <c r="R95" s="1">
+        <v>1</v>
+      </c>
+      <c r="S95" s="1">
+        <v>4</v>
+      </c>
       <c r="T95" s="1"/>
       <c r="U95" s="1"/>
       <c r="V95" s="2" t="s">
-        <v>324</v>
+        <v>38</v>
       </c>
       <c r="W95" s="2" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="X95" s="2" t="s">
         <v>239</v>
       </c>
       <c r="Y95" s="2" t="s">
+        <v>344</v>
+      </c>
+      <c r="Z95" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="AA95" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="AB95" s="2" t="s">
         <v>346</v>
-      </c>
-      <c r="Z95" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="AA95" s="2" t="s">
-        <v>328</v>
-      </c>
-      <c r="AB95" s="2" t="s">
-        <v>348</v>
       </c>
     </row>
     <row r="96" spans="1:28">
@@ -8866,16 +8930,28 @@
         <v>95</v>
       </c>
       <c r="C96" s="2" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="D96" s="2"/>
-      <c r="E96" s="1"/>
-      <c r="F96" s="2"/>
-      <c r="G96" s="2"/>
+      <c r="E96" s="1">
+        <v>37</v>
+      </c>
+      <c r="F96" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="G96" s="2" t="s">
+        <v>186</v>
+      </c>
       <c r="H96" s="2"/>
-      <c r="I96" s="1"/>
-      <c r="J96" s="2"/>
-      <c r="K96" s="2"/>
+      <c r="I96" s="1">
+        <v>26</v>
+      </c>
+      <c r="J96" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="K96" s="2" t="s">
+        <v>155</v>
+      </c>
       <c r="L96" s="2"/>
       <c r="M96" s="1">
         <v>17</v>
@@ -8890,32 +8966,36 @@
         <v>65</v>
       </c>
       <c r="Q96" s="2" t="s">
-        <v>349</v>
-      </c>
-      <c r="R96" s="1"/>
-      <c r="S96" s="1"/>
+        <v>347</v>
+      </c>
+      <c r="R96" s="1">
+        <v>0</v>
+      </c>
+      <c r="S96" s="1">
+        <v>1</v>
+      </c>
       <c r="T96" s="1"/>
       <c r="U96" s="1"/>
       <c r="V96" s="2" t="s">
-        <v>324</v>
+        <v>348</v>
       </c>
       <c r="W96" s="2" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="X96" s="2" t="s">
         <v>149</v>
       </c>
       <c r="Y96" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="Z96" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="AA96" s="2" t="s">
         <v>351</v>
       </c>
-      <c r="Z96" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="AA96" s="2" t="s">
-        <v>328</v>
-      </c>
       <c r="AB96" s="2" t="s">
-        <v>347</v>
+        <v>352</v>
       </c>
     </row>
     <row r="97" spans="1:28">
@@ -8926,16 +9006,28 @@
         <v>96</v>
       </c>
       <c r="C97" s="2" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="D97" s="2"/>
-      <c r="E97" s="1"/>
-      <c r="F97" s="2"/>
-      <c r="G97" s="2"/>
+      <c r="E97" s="1">
+        <v>7</v>
+      </c>
+      <c r="F97" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="G97" s="2" t="s">
+        <v>75</v>
+      </c>
       <c r="H97" s="2"/>
-      <c r="I97" s="1"/>
-      <c r="J97" s="2"/>
-      <c r="K97" s="2"/>
+      <c r="I97" s="1">
+        <v>43</v>
+      </c>
+      <c r="J97" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="K97" s="2" t="s">
+        <v>219</v>
+      </c>
       <c r="L97" s="2"/>
       <c r="M97" s="1">
         <v>12</v>
@@ -8950,32 +9042,32 @@
         <v>58</v>
       </c>
       <c r="Q97" s="2" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="R97" s="1"/>
       <c r="S97" s="1"/>
       <c r="T97" s="1"/>
       <c r="U97" s="1"/>
       <c r="V97" s="2" t="s">
-        <v>324</v>
+        <v>353</v>
       </c>
       <c r="W97" s="2" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="X97" s="2" t="s">
         <v>123</v>
       </c>
       <c r="Y97" s="2" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="Z97" s="2" t="s">
         <v>41</v>
       </c>
       <c r="AA97" s="2" t="s">
-        <v>328</v>
+        <v>354</v>
       </c>
       <c r="AB97" s="2" t="s">
-        <v>347</v>
+        <v>355</v>
       </c>
     </row>
     <row r="98" spans="1:28">
@@ -8986,16 +9078,28 @@
         <v>97</v>
       </c>
       <c r="C98" s="2" t="s">
-        <v>352</v>
+        <v>356</v>
       </c>
       <c r="D98" s="2"/>
-      <c r="E98" s="1"/>
-      <c r="F98" s="2"/>
-      <c r="G98" s="2"/>
+      <c r="E98" s="1">
+        <v>33</v>
+      </c>
+      <c r="F98" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="G98" s="2" t="s">
+        <v>173</v>
+      </c>
       <c r="H98" s="2"/>
-      <c r="I98" s="1"/>
-      <c r="J98" s="2"/>
-      <c r="K98" s="2"/>
+      <c r="I98" s="1">
+        <v>12</v>
+      </c>
+      <c r="J98" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="K98" s="2" t="s">
+        <v>85</v>
+      </c>
       <c r="L98" s="2"/>
       <c r="M98" s="1">
         <v>9</v>
@@ -9010,32 +9114,32 @@
         <v>65</v>
       </c>
       <c r="Q98" s="2" t="s">
-        <v>353</v>
+        <v>357</v>
       </c>
       <c r="R98" s="1"/>
       <c r="S98" s="1"/>
       <c r="T98" s="1"/>
       <c r="U98" s="1"/>
       <c r="V98" s="2" t="s">
-        <v>324</v>
+        <v>353</v>
       </c>
       <c r="W98" s="2" t="s">
-        <v>354</v>
+        <v>358</v>
       </c>
       <c r="X98" s="2" t="s">
         <v>123</v>
       </c>
       <c r="Y98" s="2" t="s">
-        <v>355</v>
+        <v>359</v>
       </c>
       <c r="Z98" s="2" t="s">
         <v>41</v>
       </c>
       <c r="AA98" s="2" t="s">
-        <v>328</v>
+        <v>354</v>
       </c>
       <c r="AB98" s="2" t="s">
-        <v>347</v>
+        <v>360</v>
       </c>
     </row>
     <row r="99" spans="1:28">
@@ -9046,16 +9150,28 @@
         <v>98</v>
       </c>
       <c r="C99" s="2" t="s">
-        <v>352</v>
+        <v>356</v>
       </c>
       <c r="D99" s="2"/>
-      <c r="E99" s="1"/>
-      <c r="F99" s="2"/>
-      <c r="G99" s="2"/>
+      <c r="E99" s="1">
+        <v>30</v>
+      </c>
+      <c r="F99" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="G99" s="2" t="s">
+        <v>142</v>
+      </c>
       <c r="H99" s="2"/>
-      <c r="I99" s="1"/>
-      <c r="J99" s="2"/>
-      <c r="K99" s="2"/>
+      <c r="I99" s="1">
+        <v>25</v>
+      </c>
+      <c r="J99" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="K99" s="2" t="s">
+        <v>153</v>
+      </c>
       <c r="L99" s="2"/>
       <c r="M99" s="1">
         <v>3</v>
@@ -9070,32 +9186,32 @@
         <v>65</v>
       </c>
       <c r="Q99" s="2" t="s">
-        <v>356</v>
+        <v>361</v>
       </c>
       <c r="R99" s="1"/>
       <c r="S99" s="1"/>
       <c r="T99" s="1"/>
       <c r="U99" s="1"/>
       <c r="V99" s="2" t="s">
-        <v>324</v>
+        <v>353</v>
       </c>
       <c r="W99" s="2" t="s">
-        <v>357</v>
+        <v>362</v>
       </c>
       <c r="X99" s="2" t="s">
         <v>40</v>
       </c>
       <c r="Y99" s="2" t="s">
-        <v>356</v>
+        <v>361</v>
       </c>
       <c r="Z99" s="2" t="s">
         <v>41</v>
       </c>
       <c r="AA99" s="2" t="s">
-        <v>328</v>
+        <v>354</v>
       </c>
       <c r="AB99" s="2" t="s">
-        <v>347</v>
+        <v>363</v>
       </c>
     </row>
     <row r="100" spans="1:28">
@@ -9106,16 +9222,28 @@
         <v>99</v>
       </c>
       <c r="C100" s="2" t="s">
-        <v>352</v>
+        <v>356</v>
       </c>
       <c r="D100" s="2"/>
-      <c r="E100" s="1"/>
-      <c r="F100" s="2"/>
-      <c r="G100" s="2"/>
+      <c r="E100" s="1">
+        <v>35</v>
+      </c>
+      <c r="F100" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="G100" s="2" t="s">
+        <v>182</v>
+      </c>
       <c r="H100" s="2"/>
-      <c r="I100" s="1"/>
-      <c r="J100" s="2"/>
-      <c r="K100" s="2"/>
+      <c r="I100" s="1">
+        <v>47</v>
+      </c>
+      <c r="J100" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="K100" s="2" t="s">
+        <v>207</v>
+      </c>
       <c r="L100" s="2"/>
       <c r="M100" s="1">
         <v>5</v>
@@ -9130,32 +9258,32 @@
         <v>65</v>
       </c>
       <c r="Q100" s="2" t="s">
-        <v>358</v>
+        <v>364</v>
       </c>
       <c r="R100" s="1"/>
       <c r="S100" s="1"/>
       <c r="T100" s="1"/>
       <c r="U100" s="1"/>
       <c r="V100" s="2" t="s">
-        <v>324</v>
+        <v>353</v>
       </c>
       <c r="W100" s="2" t="s">
-        <v>359</v>
+        <v>365</v>
       </c>
       <c r="X100" s="2" t="s">
         <v>251</v>
       </c>
       <c r="Y100" s="2" t="s">
-        <v>358</v>
+        <v>364</v>
       </c>
       <c r="Z100" s="2" t="s">
         <v>41</v>
       </c>
       <c r="AA100" s="2" t="s">
-        <v>328</v>
+        <v>354</v>
       </c>
       <c r="AB100" s="2" t="s">
-        <v>347</v>
+        <v>366</v>
       </c>
     </row>
     <row r="101" spans="1:28">
@@ -9166,7 +9294,7 @@
         <v>100</v>
       </c>
       <c r="C101" s="2" t="s">
-        <v>352</v>
+        <v>356</v>
       </c>
       <c r="D101" s="2"/>
       <c r="E101" s="1"/>
@@ -9190,32 +9318,32 @@
         <v>65</v>
       </c>
       <c r="Q101" s="2" t="s">
-        <v>358</v>
+        <v>364</v>
       </c>
       <c r="R101" s="1"/>
       <c r="S101" s="1"/>
       <c r="T101" s="1"/>
       <c r="U101" s="1"/>
       <c r="V101" s="2" t="s">
-        <v>324</v>
+        <v>353</v>
       </c>
       <c r="W101" s="2" t="s">
-        <v>359</v>
+        <v>365</v>
       </c>
       <c r="X101" s="2" t="s">
         <v>70</v>
       </c>
       <c r="Y101" s="2" t="s">
-        <v>358</v>
+        <v>364</v>
       </c>
       <c r="Z101" s="2" t="s">
         <v>41</v>
       </c>
       <c r="AA101" s="2" t="s">
-        <v>328</v>
+        <v>354</v>
       </c>
       <c r="AB101" s="2" t="s">
-        <v>347</v>
+        <v>367</v>
       </c>
     </row>
     <row r="102" spans="1:28">
@@ -9226,7 +9354,7 @@
         <v>101</v>
       </c>
       <c r="C102" s="2" t="s">
-        <v>360</v>
+        <v>368</v>
       </c>
       <c r="D102" s="2"/>
       <c r="E102" s="1"/>
@@ -9250,32 +9378,32 @@
         <v>65</v>
       </c>
       <c r="Q102" s="2" t="s">
-        <v>361</v>
+        <v>369</v>
       </c>
       <c r="R102" s="1"/>
       <c r="S102" s="1"/>
       <c r="T102" s="1"/>
       <c r="U102" s="1"/>
       <c r="V102" s="2" t="s">
-        <v>324</v>
+        <v>353</v>
       </c>
       <c r="W102" s="2" t="s">
-        <v>362</v>
+        <v>370</v>
       </c>
       <c r="X102" s="2" t="s">
         <v>40</v>
       </c>
       <c r="Y102" s="2" t="s">
-        <v>361</v>
+        <v>369</v>
       </c>
       <c r="Z102" s="2" t="s">
         <v>41</v>
       </c>
       <c r="AA102" s="2" t="s">
-        <v>328</v>
+        <v>354</v>
       </c>
       <c r="AB102" s="2" t="s">
-        <v>347</v>
+        <v>367</v>
       </c>
     </row>
     <row r="103" spans="1:28">
@@ -9286,7 +9414,7 @@
         <v>102</v>
       </c>
       <c r="C103" s="2" t="s">
-        <v>360</v>
+        <v>368</v>
       </c>
       <c r="D103" s="2"/>
       <c r="E103" s="1"/>
@@ -9310,32 +9438,32 @@
         <v>65</v>
       </c>
       <c r="Q103" s="2" t="s">
-        <v>363</v>
+        <v>371</v>
       </c>
       <c r="R103" s="1"/>
       <c r="S103" s="1"/>
       <c r="T103" s="1"/>
       <c r="U103" s="1"/>
       <c r="V103" s="2" t="s">
-        <v>324</v>
+        <v>353</v>
       </c>
       <c r="W103" s="2" t="s">
-        <v>364</v>
+        <v>372</v>
       </c>
       <c r="X103" s="2" t="s">
         <v>40</v>
       </c>
       <c r="Y103" s="2" t="s">
-        <v>363</v>
+        <v>371</v>
       </c>
       <c r="Z103" s="2" t="s">
         <v>41</v>
       </c>
       <c r="AA103" s="2" t="s">
-        <v>328</v>
+        <v>354</v>
       </c>
       <c r="AB103" s="2" t="s">
-        <v>347</v>
+        <v>367</v>
       </c>
     </row>
     <row r="104" spans="1:28">
@@ -9346,7 +9474,7 @@
         <v>103</v>
       </c>
       <c r="C104" s="2" t="s">
-        <v>365</v>
+        <v>373</v>
       </c>
       <c r="D104" s="2"/>
       <c r="E104" s="1"/>
@@ -9370,32 +9498,32 @@
         <v>65</v>
       </c>
       <c r="Q104" s="2" t="s">
-        <v>366</v>
+        <v>374</v>
       </c>
       <c r="R104" s="1"/>
       <c r="S104" s="1"/>
       <c r="T104" s="1"/>
       <c r="U104" s="1"/>
       <c r="V104" s="2" t="s">
-        <v>324</v>
+        <v>353</v>
       </c>
       <c r="W104" s="2" t="s">
-        <v>367</v>
+        <v>375</v>
       </c>
       <c r="X104" s="2" t="s">
         <v>251</v>
       </c>
       <c r="Y104" s="2" t="s">
-        <v>366</v>
+        <v>374</v>
       </c>
       <c r="Z104" s="2" t="s">
         <v>41</v>
       </c>
       <c r="AA104" s="2" t="s">
-        <v>328</v>
+        <v>354</v>
       </c>
       <c r="AB104" s="2" t="s">
-        <v>347</v>
+        <v>367</v>
       </c>
     </row>
     <row r="105" spans="1:28">
@@ -9406,7 +9534,7 @@
         <v>104</v>
       </c>
       <c r="C105" s="2" t="s">
-        <v>368</v>
+        <v>376</v>
       </c>
       <c r="D105" s="2"/>
       <c r="E105" s="1"/>
@@ -9430,32 +9558,32 @@
         <v>65</v>
       </c>
       <c r="Q105" s="2" t="s">
-        <v>369</v>
+        <v>377</v>
       </c>
       <c r="R105" s="1"/>
       <c r="S105" s="1"/>
       <c r="T105" s="1"/>
       <c r="U105" s="1"/>
       <c r="V105" s="2" t="s">
-        <v>324</v>
+        <v>353</v>
       </c>
       <c r="W105" s="2" t="s">
-        <v>370</v>
+        <v>378</v>
       </c>
       <c r="X105" s="2" t="s">
         <v>40</v>
       </c>
       <c r="Y105" s="2" t="s">
-        <v>369</v>
+        <v>377</v>
       </c>
       <c r="Z105" s="2" t="s">
         <v>41</v>
       </c>
       <c r="AA105" s="2" t="s">
-        <v>328</v>
+        <v>354</v>
       </c>
       <c r="AB105" s="2" t="s">
-        <v>347</v>
+        <v>367</v>
       </c>
     </row>
   </sheetData>

</xml_diff>